<commit_message>
agrega gráficos de burbujas y resultados finales
</commit_message>
<xml_diff>
--- a/03_Outputs/Consolidada_ref_dept/04_Cluster/Summary_Stats.xlsx
+++ b/03_Outputs/Consolidada_ref_dept/04_Cluster/Summary_Stats.xlsx
@@ -403,19 +403,19 @@
         </is>
       </c>
       <c r="C2">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D2">
-        <v>0.1854148701191617</v>
+        <v>0.2199153336754257</v>
       </c>
       <c r="E2">
-        <v>0.298644009753389</v>
+        <v>0.2572005888841792</v>
       </c>
       <c r="F2">
-        <v>-0.5390948645623808</v>
+        <v>-0.4946586428545334</v>
       </c>
       <c r="G2">
-        <v>0.5414783074640583</v>
+        <v>0.5414783074640585</v>
       </c>
     </row>
     <row r="3">
@@ -430,19 +430,19 @@
         </is>
       </c>
       <c r="C3">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3">
-        <v>-0.2434804123381046</v>
+        <v>-0.3045810299057743</v>
       </c>
       <c r="E3">
-        <v>0.5099142986554882</v>
+        <v>0.43217395488484</v>
       </c>
       <c r="F3">
-        <v>-0.9903758181507826</v>
+        <v>-0.9903758181507817</v>
       </c>
       <c r="G3">
-        <v>1.039632556582967</v>
+        <v>0.4163116189512254</v>
       </c>
     </row>
     <row r="4">
@@ -457,19 +457,19 @@
         </is>
       </c>
       <c r="C4">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D4">
-        <v>-1.148547442320373</v>
+        <v>-1.162513893310978</v>
       </c>
       <c r="E4">
-        <v>0.7528344283360701</v>
+        <v>0.7684996641586103</v>
       </c>
       <c r="F4">
-        <v>-2.568004782381657</v>
+        <v>-2.568004782381658</v>
       </c>
       <c r="G4">
-        <v>0.1098984705398998</v>
+        <v>0.1098984705398971</v>
       </c>
     </row>
     <row r="5">
@@ -484,19 +484,19 @@
         </is>
       </c>
       <c r="C5">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5">
-        <v>-0.6924701948406524</v>
+        <v>-0.6506213390103812</v>
       </c>
       <c r="E5">
-        <v>0.66699959023602</v>
+        <v>0.6532053493973999</v>
       </c>
       <c r="F5">
-        <v>-2.190101423182183</v>
+        <v>-2.190101423182182</v>
       </c>
       <c r="G5">
-        <v>0.7004613350944694</v>
+        <v>0.7004613350944741</v>
       </c>
     </row>
     <row r="6">
@@ -511,19 +511,19 @@
         </is>
       </c>
       <c r="C6">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D6">
-        <v>0.3970446375168671</v>
+        <v>0.4119476761871822</v>
       </c>
       <c r="E6">
-        <v>0.7299911022435481</v>
+        <v>0.7445809807195729</v>
       </c>
       <c r="F6">
-        <v>-0.6466707801021823</v>
+        <v>-0.6466707801021813</v>
       </c>
       <c r="G6">
-        <v>2.131288547471114</v>
+        <v>2.131288547471112</v>
       </c>
     </row>
     <row r="7">
@@ -538,19 +538,19 @@
         </is>
       </c>
       <c r="C7">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7">
-        <v>0.4852619838457546</v>
+        <v>0.4699653005788321</v>
       </c>
       <c r="E7">
-        <v>0.7273182730833765</v>
+        <v>0.7416443413731844</v>
       </c>
       <c r="F7">
-        <v>-0.8978785963052078</v>
+        <v>-0.8978785963052089</v>
       </c>
       <c r="G7">
-        <v>2.06455055072084</v>
+        <v>2.064550550720848</v>
       </c>
     </row>
     <row r="8">
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="C8">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8">
-        <v>1.258614418683842</v>
+        <v>1.31085349556562</v>
       </c>
       <c r="E8">
-        <v>0.9939076867875956</v>
+        <v>0.9870192681519995</v>
       </c>
       <c r="F8">
-        <v>-0.3461373601818123</v>
+        <v>-0.3461373601818119</v>
       </c>
       <c r="G8">
-        <v>4.171809563477858</v>
+        <v>4.171809563477855</v>
       </c>
     </row>
     <row r="9">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="C9">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9">
-        <v>-0.1434934980556117</v>
+        <v>-0.1451215070733966</v>
       </c>
       <c r="E9">
-        <v>2.332813857497649</v>
+        <v>2.390410068141249</v>
       </c>
       <c r="F9">
         <v>-1.335422301040694</v>
@@ -619,19 +619,19 @@
         </is>
       </c>
       <c r="C10">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D10">
-        <v>0.7835514721166872</v>
+        <v>0.7911484674096021</v>
       </c>
       <c r="E10">
-        <v>0.3230779112308435</v>
+        <v>0.3290366276962908</v>
       </c>
       <c r="F10">
-        <v>0.04078424802624479</v>
+        <v>0.04078424802624404</v>
       </c>
       <c r="G10">
-        <v>1.415016166418096</v>
+        <v>1.415016166418095</v>
       </c>
     </row>
     <row r="11">
@@ -646,19 +646,19 @@
         </is>
       </c>
       <c r="C11">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D11">
-        <v>0.5875009209166207</v>
+        <v>0.6205637558335411</v>
       </c>
       <c r="E11">
-        <v>0.5013722637526776</v>
+        <v>0.4885601957641811</v>
       </c>
       <c r="F11">
-        <v>-0.2431724151910864</v>
+        <v>-0.2431724151910867</v>
       </c>
       <c r="G11">
-        <v>1.355836895456324</v>
+        <v>1.355836895456326</v>
       </c>
     </row>
     <row r="12">
@@ -673,16 +673,16 @@
         </is>
       </c>
       <c r="C12">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D12">
-        <v>1.220826587031085</v>
+        <v>1.205053005970531</v>
       </c>
       <c r="E12">
-        <v>1.179485790408179</v>
+        <v>1.206233248965432</v>
       </c>
       <c r="F12">
-        <v>-0.2514776451064171</v>
+        <v>-0.2514776451064176</v>
       </c>
       <c r="G12">
         <v>3.96815963947509</v>
@@ -700,19 +700,19 @@
         </is>
       </c>
       <c r="C13">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D13">
-        <v>0.8308470844150752</v>
+        <v>0.8329693711842878</v>
       </c>
       <c r="E13">
-        <v>1.365851249250529</v>
+        <v>1.39954388001844</v>
       </c>
       <c r="F13">
         <v>-1.381721156492645</v>
       </c>
       <c r="G13">
-        <v>3.361539269928816</v>
+        <v>3.361539269928818</v>
       </c>
     </row>
     <row r="14">
@@ -727,19 +727,19 @@
         </is>
       </c>
       <c r="C14">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D14">
-        <v>-0.6126767551128059</v>
+        <v>-0.6217778737700066</v>
       </c>
       <c r="E14">
-        <v>0.4898324055057766</v>
+        <v>0.5000191930546143</v>
       </c>
       <c r="F14">
-        <v>-1.699620576629202</v>
+        <v>-1.699620576629203</v>
       </c>
       <c r="G14">
-        <v>0.03536957885062039</v>
+        <v>0.03536957885062244</v>
       </c>
     </row>
     <row r="15">
@@ -754,19 +754,19 @@
         </is>
       </c>
       <c r="C15">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D15">
-        <v>-0.4513347755991502</v>
+        <v>-0.4363848686364001</v>
       </c>
       <c r="E15">
-        <v>0.8372731197968304</v>
+        <v>0.8549355224230254</v>
       </c>
       <c r="F15">
-        <v>-1.766259700036685</v>
+        <v>-1.766259700036686</v>
       </c>
       <c r="G15">
-        <v>0.8290671596956763</v>
+        <v>0.829067159695676</v>
       </c>
     </row>
     <row r="16">
@@ -781,16 +781,16 @@
         </is>
       </c>
       <c r="C16">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D16">
-        <v>1.299404630505814</v>
+        <v>1.301941301202025</v>
       </c>
       <c r="E16">
-        <v>0.6403797947609478</v>
+        <v>0.6560807527172793</v>
       </c>
       <c r="F16">
-        <v>-0.3460087464425586</v>
+        <v>-0.3460087464425587</v>
       </c>
       <c r="G16">
         <v>2.346393885941261</v>
@@ -808,19 +808,19 @@
         </is>
       </c>
       <c r="C17">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17">
-        <v>0.1820941706032099</v>
+        <v>0.2132669952141425</v>
       </c>
       <c r="E17">
-        <v>0.5013107472777508</v>
+        <v>0.4913560615647438</v>
       </c>
       <c r="F17">
-        <v>-0.5931843066935157</v>
+        <v>-0.593184306693515</v>
       </c>
       <c r="G17">
-        <v>1.34486131205115</v>
+        <v>1.344861312051155</v>
       </c>
     </row>
     <row r="18">
@@ -835,19 +835,19 @@
         </is>
       </c>
       <c r="C18">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D18">
-        <v>-1.271106253768265</v>
+        <v>-1.308664770562603</v>
       </c>
       <c r="E18">
-        <v>0.601925317772898</v>
+        <v>0.5897829754572792</v>
       </c>
       <c r="F18">
-        <v>-2.79908406316295</v>
+        <v>-2.799084063162949</v>
       </c>
       <c r="G18">
-        <v>-0.4823774010871604</v>
+        <v>-0.4942603480178074</v>
       </c>
     </row>
     <row r="19">
@@ -862,16 +862,16 @@
         </is>
       </c>
       <c r="C19">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D19">
-        <v>0.0160716834609138</v>
+        <v>0.02775304689534336</v>
       </c>
       <c r="E19">
-        <v>0.8236472972263404</v>
+        <v>0.8421178780465908</v>
       </c>
       <c r="F19">
-        <v>-1.982969290230687</v>
+        <v>-1.982969290230689</v>
       </c>
       <c r="G19">
         <v>1.308361824367727</v>
@@ -889,19 +889,19 @@
         </is>
       </c>
       <c r="C20">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D20">
-        <v>0.2936422101065232</v>
+        <v>0.2797294819517756</v>
       </c>
       <c r="E20">
-        <v>0.4855516968598177</v>
+        <v>0.4930285431198367</v>
       </c>
       <c r="F20">
-        <v>-0.8085156722433736</v>
+        <v>-0.8085156722433759</v>
       </c>
       <c r="G20">
-        <v>1.029358337896933</v>
+        <v>1.029358337896934</v>
       </c>
     </row>
     <row r="21">
@@ -916,19 +916,19 @@
         </is>
       </c>
       <c r="C21">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D21">
-        <v>1.335568411274081</v>
+        <v>1.388390932652582</v>
       </c>
       <c r="E21">
-        <v>0.7195645043434036</v>
+        <v>0.6922482764442586</v>
       </c>
       <c r="F21">
-        <v>0.08475956622982121</v>
+        <v>0.0847595662298201</v>
       </c>
       <c r="G21">
-        <v>2.827916595898227</v>
+        <v>2.827916595898226</v>
       </c>
     </row>
     <row r="22">
@@ -943,19 +943,19 @@
         </is>
       </c>
       <c r="C22">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D22">
-        <v>-0.316743539333204</v>
+        <v>-0.3315134946245369</v>
       </c>
       <c r="E22">
-        <v>0.6593561311949463</v>
+        <v>0.6718993463678711</v>
       </c>
       <c r="F22">
         <v>-1.585043690497099</v>
       </c>
       <c r="G22">
-        <v>1.027923311020653</v>
+        <v>1.027923311020652</v>
       </c>
     </row>
     <row r="23">
@@ -970,19 +970,19 @@
         </is>
       </c>
       <c r="C23">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D23">
-        <v>-0.1955830265152131</v>
+        <v>-0.2385175712607449</v>
       </c>
       <c r="E23">
-        <v>0.7179530853091849</v>
+        <v>0.706149770784734</v>
       </c>
       <c r="F23">
-        <v>-1.537758853224991</v>
+        <v>-1.537758853224986</v>
       </c>
       <c r="G23">
-        <v>1.137188722282123</v>
+        <v>1.13718872228213</v>
       </c>
     </row>
     <row r="24">
@@ -997,19 +997,19 @@
         </is>
       </c>
       <c r="C24">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D24">
-        <v>-0.3192666710001147</v>
+        <v>-0.3252090331472903</v>
       </c>
       <c r="E24">
-        <v>1.001930669693688</v>
+        <v>1.026276093791661</v>
       </c>
       <c r="F24">
-        <v>-3.378910429378913</v>
+        <v>-3.378910429378875</v>
       </c>
       <c r="G24">
-        <v>1.42728657404968</v>
+        <v>1.427286574049681</v>
       </c>
     </row>
     <row r="25">
@@ -1024,13 +1024,13 @@
         </is>
       </c>
       <c r="C25">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D25">
-        <v>0.9986943913408779</v>
+        <v>1.014454530658547</v>
       </c>
       <c r="E25">
-        <v>0.4472974100469918</v>
+        <v>0.4520410354018418</v>
       </c>
       <c r="F25">
         <v>0.3887221707351368</v>
@@ -1051,19 +1051,19 @@
         </is>
       </c>
       <c r="C26">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D26">
-        <v>-0.5600273587810581</v>
+        <v>-0.5177194850105131</v>
       </c>
       <c r="E26">
-        <v>0.723829019669869</v>
+        <v>0.7132859765725932</v>
       </c>
       <c r="F26">
-        <v>-2.054611080772094</v>
+        <v>-2.054611080772093</v>
       </c>
       <c r="G26">
-        <v>0.6156397183774129</v>
+        <v>0.6156397183774134</v>
       </c>
     </row>
     <row r="27">
@@ -1078,19 +1078,19 @@
         </is>
       </c>
       <c r="C27">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D27">
-        <v>0.5387048081561651</v>
+        <v>0.5383558628534768</v>
       </c>
       <c r="E27">
-        <v>0.05741442860925543</v>
+        <v>0.05880837288952247</v>
       </c>
       <c r="F27">
-        <v>0.4561999031069825</v>
+        <v>0.4561999031069822</v>
       </c>
       <c r="G27">
-        <v>0.6742770223226823</v>
+        <v>0.674277022322684</v>
       </c>
     </row>
     <row r="28">
@@ -1105,16 +1105,16 @@
         </is>
       </c>
       <c r="C28">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D28">
-        <v>0.691246888809454</v>
+        <v>0.6690136766761482</v>
       </c>
       <c r="E28">
-        <v>1.227125204988511</v>
+        <v>1.252880436825972</v>
       </c>
       <c r="F28">
-        <v>-0.5523795259463992</v>
+        <v>-0.5523795259463995</v>
       </c>
       <c r="G28">
         <v>3.473744060831262</v>
@@ -1132,16 +1132,16 @@
         </is>
       </c>
       <c r="C29">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D29">
-        <v>0.6613905421790905</v>
+        <v>0.6903052863484477</v>
       </c>
       <c r="E29">
-        <v>1.089912227512826</v>
+        <v>1.108147578043784</v>
       </c>
       <c r="F29">
-        <v>-0.9174599709233661</v>
+        <v>-0.9174599709233657</v>
       </c>
       <c r="G29">
         <v>3.031169374090164</v>
@@ -1159,16 +1159,16 @@
         </is>
       </c>
       <c r="C30">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D30">
-        <v>0.4776337877444925</v>
+        <v>0.492470812368887</v>
       </c>
       <c r="E30">
-        <v>0.584175500621073</v>
+        <v>0.5943390401773995</v>
       </c>
       <c r="F30">
-        <v>-0.5819640447251712</v>
+        <v>-0.5819640447251709</v>
       </c>
       <c r="G30">
         <v>2.347056830336199</v>
@@ -1186,16 +1186,16 @@
         </is>
       </c>
       <c r="C31">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D31">
-        <v>0.6348285613796906</v>
+        <v>0.6526734231642003</v>
       </c>
       <c r="E31">
-        <v>0.3932780016223138</v>
+        <v>0.3937575686388039</v>
       </c>
       <c r="F31">
-        <v>-0.01542661154383375</v>
+        <v>-0.01542661154383271</v>
       </c>
       <c r="G31">
         <v>1.321121714849001</v>
@@ -1213,19 +1213,19 @@
         </is>
       </c>
       <c r="C32">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D32">
-        <v>1.016502330973626</v>
+        <v>1.048109451515631</v>
       </c>
       <c r="E32">
-        <v>0.9400637723024254</v>
+        <v>0.9512248725734297</v>
       </c>
       <c r="F32">
-        <v>-0.347104406105941</v>
+        <v>-0.3471044061059401</v>
       </c>
       <c r="G32">
-        <v>2.959130920088872</v>
+        <v>2.959130920088874</v>
       </c>
     </row>
     <row r="33">
@@ -1240,19 +1240,19 @@
         </is>
       </c>
       <c r="C33">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D33">
-        <v>0.4647134284915202</v>
+        <v>0.4375226067510983</v>
       </c>
       <c r="E33">
-        <v>0.5689203394056236</v>
+        <v>0.5662491696667651</v>
       </c>
       <c r="F33">
-        <v>-0.5790684254232037</v>
+        <v>-0.6055941961081263</v>
       </c>
       <c r="G33">
-        <v>1.580006566982992</v>
+        <v>1.545326930774329</v>
       </c>
     </row>
   </sheetData>

</xml_diff>